<commit_message>
Formalize the third Anki export pathway (multi-card conditional note type)
README gains 'Exporting to Anki - the three pathways' with the hand-built
import from the video credited in the original tuto: tab-delimited UTF-8 txt,
cloned note type with fields in column order, conditional card templates that
skip blanks, and matrix-specific front/back examples. Same steps condensed
into the workbook tuto tab; the '10 Question' template is noted as absent
from the repo with recreate-or-download guidance.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R1F9PpTbWP4vggx6q7LbDZ
</commit_message>
<xml_diff>
--- a/00.Memory_systems/06.Programming_Millenium/Programming_Millenium.xlsx
+++ b/00.Memory_systems/06.Programming_Millenium/Programming_Millenium.xlsx
@@ -51426,7 +51426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C9"/>
+  <dimension ref="A2:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -51538,17 +51538,107 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3rd way</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>excel</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>multi-card import (see README 'Pathway 3'): save the matrix tab as tab-delimited .txt, re-saved as UTF-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3rd way</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>anki</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>manage note types -&gt; clone Basic (the '10 Question' type is not in the repo - recreating it IS these steps) -&gt; fields = Code, Concept, Anchor, Definition, Example, Confusables IN COLUMN ORDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3rd way</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>anki</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>cards: one template per question, front wrapped in a conditional so blanks make no card: {{#Definition}}Definition of {{Code}} {{Concept}}?{{/Definition}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3rd way</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>anki</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>back: {{FrontSide}} &lt;hr id=answer&gt; {{Definition}} - repeat per column; reverse card {{#Concept}}Address of {{Concept}}?{{/Concept}} -&gt; {{Code}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3rd way</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>anki</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>file -&gt; import the .txt (separator Tab, note type = the clone, fields map in order); each note yields one card per non-blank template</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>more advanced</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>youtube</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Converting a COMPLEX Excel file to an Anki deck! - YouTube</t>
         </is>

</xml_diff>